<commit_message>
Muestra: categorías reales en el input 1
La columna Categoría traía el segmento (Soluciones / Ingredientes). El input
real trae Café, Chocolatería, etc., que es sobre lo que se arman las reglas.
Derivada del producto, sin tocar el azar: la base y el input 2 dan los
mismos bytes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sample/input1_objetivo.xlsx
+++ b/data/sample/input1_objetivo.xlsx
@@ -463,7 +463,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -492,7 +492,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -579,7 +579,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -608,7 +608,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Lácteos</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -637,7 +637,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -724,7 +724,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Lácteos</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -753,7 +753,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -782,7 +782,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Lácteos</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -840,7 +840,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Lácteos</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -869,7 +869,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -898,7 +898,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Culinarios</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -956,7 +956,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -985,7 +985,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Chocolatería</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1072,7 +1072,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1130,7 +1130,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1188,7 +1188,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1246,7 +1246,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1275,7 +1275,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1304,7 +1304,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1333,7 +1333,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1362,7 +1362,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1391,7 +1391,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Vajilla</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1420,7 +1420,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1449,7 +1449,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1478,7 +1478,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Vajilla</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1507,7 +1507,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1565,7 +1565,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Vajilla</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1594,7 +1594,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Endulzantes</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1623,7 +1623,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Vajilla</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1652,7 +1652,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Vajilla</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1710,7 +1710,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Descartables</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1768,7 +1768,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Soluciones</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1797,7 +1797,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Lácteos</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1826,7 +1826,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ingredientes</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">

</xml_diff>